<commit_message>
Adiciona Excel formatado gerado automaticamente
</commit_message>
<xml_diff>
--- a/scripts/excel/sdg-data-formatado.xlsx
+++ b/scripts/excel/sdg-data-formatado.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -510,7 +510,7 @@
       <c r="C2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="4" t="inlineStr"/>
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
@@ -527,6 +527,7 @@
       <c r="C3" t="n">
         <v>3</v>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" t="n">
@@ -540,6 +541,7 @@
       <c r="C4" t="n">
         <v>2</v>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" t="n">
@@ -553,6 +555,7 @@
       <c r="C5" t="n">
         <v>1</v>
       </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" t="n">
@@ -566,6 +569,7 @@
       <c r="C6" t="n">
         <v>3</v>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" t="n">
@@ -579,6 +583,7 @@
       <c r="C7" t="n">
         <v>2</v>
       </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" t="n">
@@ -592,6 +597,7 @@
       <c r="C8" t="n">
         <v>3</v>
       </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" t="n">
@@ -605,6 +611,7 @@
       <c r="C9" t="n">
         <v>1</v>
       </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" t="n">
@@ -618,55 +625,78 @@
       <c r="C10" t="n">
         <v>2</v>
       </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="n">
+        <v>60</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" t="inlineStr">
         <is>
           <t>SDGindicator: indicator</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="25" customHeight="1">
-      <c r="A12" t="inlineStr">
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Metric and indicator reference</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Metric / Indicator</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Value
 (for continuous data)</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Yes/No</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Public
 (Yes/No)</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="25" customHeight="1"/>
-    <row r="14" ht="25" customHeight="1"/>
     <row r="15" ht="25" customHeight="1"/>
     <row r="16" ht="25" customHeight="1"/>
     <row r="17" ht="25" customHeight="1"/>

</xml_diff>